<commit_message>
docs(use-cases): use role names and EnergyMonitor in tables and diagrams
</commit_message>
<xml_diff>
--- a/Diagramas de casos de uso/Diagramas de casos de uso/Tablas descripcion caso de uso.xlsx
+++ b/Diagramas de casos de uso/Diagramas de casos de uso/Tablas descripcion caso de uso.xlsx
@@ -509,6 +509,8 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
@@ -594,7 +596,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Usuario (OWNER)</t>
+          <t>Usuario (propietario)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -614,7 +616,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Asigna OWNER al usuario creador y MEMBER a los usuarios vinculados al proyecto.</t>
+          <t>Asigna el rol de propietario al usuario creador y el de miembro a los usuarios vinculados al proyecto.</t>
         </is>
       </c>
     </row>
@@ -626,7 +628,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Usuario (OWNER)</t>
+          <t>Usuario (propietario)</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -635,6 +637,8 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
@@ -741,6 +745,8 @@
     <row r="31">
       <c r="A31" s="1" t="n"/>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
@@ -796,7 +802,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Usuario (OWNER/MEMBER)</t>
+          <t>Usuario (propietario/miembro)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -871,7 +877,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Usuario (OWNER/MEMBER)</t>
+          <t>Usuario (propietario/miembro)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -913,7 +919,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Usuario (OWNER)</t>
+          <t>Usuario (propietario)</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">

</xml_diff>